<commit_message>
240105 - finalised contreras huerta code
FIXES:
- softmax function includes bias parameter for constantino & daw models
- buildData simplified and reads in block order
- estimates reinitialised per block (simplest to write in the code)
- fitting_240104 contains new test fitting data for models 1, 5-10. Results look the same
</commit_message>
<xml_diff>
--- a/model/foragingModelTable.xlsx
+++ b/model/foragingModelTable.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11008"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11210"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/exs165/Dropbox/foraging/stochastic-mvt-project/model/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4C848007-5036-2849-BF4A-D392C6542052}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1A1487CA-6407-5241-BF6B-4E556C624CE8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="460" yWindow="500" windowWidth="27240" windowHeight="16320" xr2:uid="{AF09A64C-08B3-A642-B0D0-C38CF1EBFD20}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="81" uniqueCount="21">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="82" uniqueCount="22">
   <si>
     <t>softmax</t>
   </si>
@@ -99,6 +99,9 @@
   </si>
   <si>
     <t>twoScalar</t>
+  </si>
+  <si>
+    <t>bias</t>
   </si>
 </sst>
 </file>
@@ -458,10 +461,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{766F6688-A436-6A43-9B8F-A83A43AD55B0}">
-  <dimension ref="A1:F26"/>
+  <dimension ref="A1:G26"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>9</v>
       </c>
@@ -480,8 +483,11 @@
       <c r="F1" t="s">
         <v>15</v>
       </c>
-    </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="G1" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A2">
         <v>1</v>
       </c>
@@ -500,8 +506,11 @@
       <c r="F2" t="s">
         <v>14</v>
       </c>
-    </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="G2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A3">
         <v>2</v>
       </c>
@@ -520,8 +529,11 @@
       <c r="F3" t="s">
         <v>14</v>
       </c>
-    </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="G3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A4">
         <v>3</v>
       </c>
@@ -540,8 +552,11 @@
       <c r="F4" t="s">
         <v>14</v>
       </c>
-    </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="G4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A5">
         <v>4</v>
       </c>
@@ -560,8 +575,11 @@
       <c r="F5" t="s">
         <v>14</v>
       </c>
-    </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="G5">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A6">
         <v>5</v>
       </c>
@@ -578,10 +596,13 @@
         <v>3</v>
       </c>
       <c r="F6" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.2">
+        <v>6</v>
+      </c>
+      <c r="G6">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A7">
         <v>6</v>
       </c>
@@ -598,10 +619,13 @@
         <v>3</v>
       </c>
       <c r="F7" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.2">
+        <v>6</v>
+      </c>
+      <c r="G7">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A8">
         <v>7</v>
       </c>
@@ -618,10 +642,13 @@
         <v>3</v>
       </c>
       <c r="F8" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.2">
+        <v>6</v>
+      </c>
+      <c r="G8">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A9">
         <v>8</v>
       </c>
@@ -640,8 +667,11 @@
       <c r="F9" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="G9">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A10">
         <v>9</v>
       </c>
@@ -660,8 +690,11 @@
       <c r="F10" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="G10">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A11">
         <v>10</v>
       </c>
@@ -680,8 +713,11 @@
       <c r="F11" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="G11">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A12">
         <v>11</v>
       </c>
@@ -700,8 +736,11 @@
       <c r="F12" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="G12">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A13">
         <v>12</v>
       </c>
@@ -720,8 +759,11 @@
       <c r="F13" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="G13">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A14">
         <v>13</v>
       </c>
@@ -740,8 +782,11 @@
       <c r="F14" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="G14">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A15">
         <v>14</v>
       </c>
@@ -760,8 +805,11 @@
       <c r="F15" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="G15">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A16">
         <v>15</v>
       </c>
@@ -780,8 +828,11 @@
       <c r="F16" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="G16">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="17" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A17">
         <v>16</v>
       </c>
@@ -800,8 +851,11 @@
       <c r="F17" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="G17">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="18" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A18">
         <v>17</v>
       </c>
@@ -820,8 +874,11 @@
       <c r="F18" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="G18">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="19" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A19">
         <v>18</v>
       </c>
@@ -840,8 +897,11 @@
       <c r="F19" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="G19">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="20" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A20">
         <v>19</v>
       </c>
@@ -860,8 +920,11 @@
       <c r="F20" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="G20">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="21" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A21">
         <v>20</v>
       </c>
@@ -880,8 +943,11 @@
       <c r="F21" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="22" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="G21">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="22" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A22">
         <v>21</v>
       </c>
@@ -900,8 +966,11 @@
       <c r="F22" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="23" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="G22">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="23" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A23">
         <v>22</v>
       </c>
@@ -920,8 +989,11 @@
       <c r="F23" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="24" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="G23">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="24" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A24">
         <v>23</v>
       </c>
@@ -940,8 +1012,11 @@
       <c r="F24" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="25" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="G24">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="25" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A25">
         <v>24</v>
       </c>
@@ -960,8 +1035,11 @@
       <c r="F25" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="26" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="G25">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="26" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A26">
         <v>25</v>
       </c>
@@ -979,6 +1057,9 @@
       </c>
       <c r="F26" t="s">
         <v>8</v>
+      </c>
+      <c r="G26">
+        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
UPDATE: fitting beta models
</commit_message>
<xml_diff>
--- a/model/foragingModelTable.xlsx
+++ b/model/foragingModelTable.xlsx
@@ -8,14 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/exs165/Dropbox/foraging/stochastic-mvt-project/model/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1C06858F-8C9B-984A-9453-219175C0EDE4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E1887B2D-6A71-A24C-BADC-F5CF4CE275AD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="500" windowWidth="28800" windowHeight="16320" xr2:uid="{AF09A64C-08B3-A642-B0D0-C38CF1EBFD20}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="181029"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -36,14 +36,11 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="99" uniqueCount="21">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="63" uniqueCount="18">
   <si>
     <t>softmax</t>
   </si>
   <si>
-    <t>twoExponential</t>
-  </si>
-  <si>
     <t>exponential</t>
   </si>
   <si>
@@ -80,13 +77,7 @@
     <t>hyperbolic</t>
   </si>
   <si>
-    <t>twoHyperbolic</t>
-  </si>
-  <si>
     <t>scalar</t>
-  </si>
-  <si>
-    <t>twoScalar</t>
   </si>
   <si>
     <t>bias</t>
@@ -458,30 +449,30 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{766F6688-A436-6A43-9B8F-A83A43AD55B0}">
-  <dimension ref="A1:G24"/>
+  <dimension ref="A1:G15"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
+        <v>5</v>
+      </c>
+      <c r="B1" t="s">
         <v>6</v>
       </c>
-      <c r="B1" t="s">
+      <c r="C1" t="s">
+        <v>11</v>
+      </c>
+      <c r="D1" t="s">
         <v>7</v>
       </c>
-      <c r="C1" t="s">
-        <v>12</v>
-      </c>
-      <c r="D1" t="s">
+      <c r="E1" t="s">
         <v>8</v>
       </c>
-      <c r="E1" t="s">
-        <v>9</v>
-      </c>
       <c r="F1" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="G1" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.2">
@@ -498,13 +489,13 @@
         <v>0</v>
       </c>
       <c r="E2" t="s">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="F2" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="G2" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.2">
@@ -521,13 +512,13 @@
         <v>0</v>
       </c>
       <c r="E3" t="s">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="F3" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="G3" t="s">
-        <v>18</v>
+        <v>15</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.2">
@@ -544,13 +535,13 @@
         <v>0</v>
       </c>
       <c r="E4" t="s">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="F4" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="G4" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.2">
@@ -567,13 +558,13 @@
         <v>0</v>
       </c>
       <c r="E5" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="F5" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="G5" t="s">
-        <v>18</v>
+        <v>15</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.2">
@@ -590,13 +581,13 @@
         <v>0</v>
       </c>
       <c r="E6" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="F6" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="G6" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.2">
@@ -613,13 +604,13 @@
         <v>0</v>
       </c>
       <c r="E7" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="F7" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G7" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.2">
@@ -636,13 +627,13 @@
         <v>0</v>
       </c>
       <c r="E8" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="F8" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="G8" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.2">
@@ -659,13 +650,13 @@
         <v>0</v>
       </c>
       <c r="E9" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="F9" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="G9" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.2">
@@ -682,13 +673,13 @@
         <v>0</v>
       </c>
       <c r="E10" t="s">
+        <v>1</v>
+      </c>
+      <c r="F10" t="s">
         <v>2</v>
       </c>
-      <c r="F10" t="s">
-        <v>3</v>
-      </c>
       <c r="G10" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.2">
@@ -705,13 +696,13 @@
         <v>0</v>
       </c>
       <c r="E11" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F11" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="G11" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.2">
@@ -728,13 +719,13 @@
         <v>0</v>
       </c>
       <c r="E12" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F12" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="G12" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.2">
@@ -751,13 +742,13 @@
         <v>0</v>
       </c>
       <c r="E13" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="F13" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G13" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.2">
@@ -774,13 +765,13 @@
         <v>0</v>
       </c>
       <c r="E14" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="F14" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="G14" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.2">
@@ -797,220 +788,13 @@
         <v>0</v>
       </c>
       <c r="E15" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="F15" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="G15" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A16">
-        <v>15</v>
-      </c>
-      <c r="B16" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="C16">
-        <v>0</v>
-      </c>
-      <c r="D16">
-        <v>0</v>
-      </c>
-      <c r="E16" t="s">
-        <v>16</v>
-      </c>
-      <c r="F16" t="s">
-        <v>3</v>
-      </c>
-      <c r="G16" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="17" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A17">
-        <v>16</v>
-      </c>
-      <c r="B17" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="C17">
-        <v>0</v>
-      </c>
-      <c r="D17">
-        <v>0</v>
-      </c>
-      <c r="E17" t="s">
-        <v>16</v>
-      </c>
-      <c r="F17" t="s">
-        <v>4</v>
-      </c>
-      <c r="G17" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="18" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A18">
-        <v>17</v>
-      </c>
-      <c r="B18" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="C18">
-        <v>1</v>
-      </c>
-      <c r="D18">
-        <v>0</v>
-      </c>
-      <c r="E18" t="s">
-        <v>16</v>
-      </c>
-      <c r="F18" t="s">
-        <v>5</v>
-      </c>
-      <c r="G18" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="19" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A19">
-        <v>18</v>
-      </c>
-      <c r="B19" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="C19">
-        <v>0</v>
-      </c>
-      <c r="D19">
-        <v>0</v>
-      </c>
-      <c r="E19" t="s">
-        <v>1</v>
-      </c>
-      <c r="F19" t="s">
-        <v>3</v>
-      </c>
-      <c r="G19" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="20" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A20">
-        <v>19</v>
-      </c>
-      <c r="B20" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="C20">
-        <v>0</v>
-      </c>
-      <c r="D20">
-        <v>0</v>
-      </c>
-      <c r="E20" t="s">
-        <v>1</v>
-      </c>
-      <c r="F20" t="s">
-        <v>4</v>
-      </c>
-      <c r="G20" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="21" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A21">
-        <v>20</v>
-      </c>
-      <c r="B21" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="C21">
-        <v>1</v>
-      </c>
-      <c r="D21">
-        <v>0</v>
-      </c>
-      <c r="E21" t="s">
-        <v>1</v>
-      </c>
-      <c r="F21" t="s">
-        <v>5</v>
-      </c>
-      <c r="G21" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="22" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A22">
-        <v>21</v>
-      </c>
-      <c r="B22" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="C22">
-        <v>0</v>
-      </c>
-      <c r="D22">
-        <v>0</v>
-      </c>
-      <c r="E22" t="s">
-        <v>14</v>
-      </c>
-      <c r="F22" t="s">
-        <v>3</v>
-      </c>
-      <c r="G22" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="23" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A23">
-        <v>22</v>
-      </c>
-      <c r="B23" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="C23">
-        <v>0</v>
-      </c>
-      <c r="D23">
-        <v>0</v>
-      </c>
-      <c r="E23" t="s">
-        <v>14</v>
-      </c>
-      <c r="F23" t="s">
-        <v>4</v>
-      </c>
-      <c r="G23" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="24" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A24">
-        <v>23</v>
-      </c>
-      <c r="B24" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="C24">
-        <v>1</v>
-      </c>
-      <c r="D24">
-        <v>0</v>
-      </c>
-      <c r="E24" t="s">
-        <v>14</v>
-      </c>
-      <c r="F24" t="s">
-        <v>5</v>
-      </c>
-      <c r="G24" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
     </row>
   </sheetData>

</xml_diff>